<commit_message>
add actions to excl
</commit_message>
<xml_diff>
--- a/docs/cms-changes.xlsx
+++ b/docs/cms-changes.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K42"/>
+  <dimension ref="A1:K44"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1476,7 +1476,7 @@
         <v>0</v>
       </c>
       <c r="I31" t="str">
-        <v>move_items_to_part</v>
+        <v>פיצול/העברה מ-2011060</v>
       </c>
       <c r="J31" t="str">
         <v>כן</v>
@@ -1861,7 +1861,7 @@
         <v>0</v>
       </c>
       <c r="I42" t="str">
-        <v>update_part</v>
+        <v>עדכון שם: פרשת העקידה</v>
       </c>
       <c r="J42" t="str">
         <v>כן</v>
@@ -1870,16 +1870,86 @@
         <v/>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>chg_1773733140069_rtmbazn</v>
+      </c>
+      <c r="B43" t="str">
+        <v>17.3.2026, 9:39:00</v>
+      </c>
+      <c r="C43" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D43" t="str">
+        <v>edot_mizrah</v>
+      </c>
+      <c r="E43" t="str">
+        <v>0-edot_mizrah</v>
+      </c>
+      <c r="F43" t="str">
+        <v>3015010</v>
+      </c>
+      <c r="G43" t="str">
+        <v>3011035</v>
+      </c>
+      <c r="H43">
+        <v>1</v>
+      </c>
+      <c r="I43" t="str">
+        <v>1 שינוי שדה</v>
+      </c>
+      <c r="J43" t="str">
+        <v>כן</v>
+      </c>
+      <c r="K43" t="str">
+        <v>לא</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>chg_1773733142825_6uxc5ua</v>
+      </c>
+      <c r="B44" t="str">
+        <v>17.3.2026, 9:39:02</v>
+      </c>
+      <c r="C44" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D44" t="str">
+        <v>edot_mizrah</v>
+      </c>
+      <c r="E44" t="str">
+        <v/>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <v/>
+      </c>
+      <c r="H44">
+        <v>0</v>
+      </c>
+      <c r="I44" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="J44" t="str">
+        <v>כן</v>
+      </c>
+      <c r="K44" t="str">
+        <v>כן</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K42"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K44"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O164"/>
+  <dimension ref="A1:O167"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -9589,9 +9659,151 @@
         <v>V</v>
       </c>
     </row>
+    <row r="165">
+      <c r="A165" t="str">
+        <v>chg_1773665935976_g4os2pm</v>
+      </c>
+      <c r="B165" t="str">
+        <v>16.3.2026, 14:58:55</v>
+      </c>
+      <c r="C165" t="str">
+        <v>update_part</v>
+      </c>
+      <c r="D165" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="E165" t="str">
+        <v>0-sefard</v>
+      </c>
+      <c r="F165" t="str">
+        <v/>
+      </c>
+      <c r="G165" t="str">
+        <v>2015010</v>
+      </c>
+      <c r="H165" t="str">
+        <v>פרשת העקידה</v>
+      </c>
+      <c r="I165" t="str">
+        <v>2011821</v>
+      </c>
+      <c r="J165" t="str">
+        <v/>
+      </c>
+      <c r="K165" t="str">
+        <v/>
+      </c>
+      <c r="L165" t="str">
+        <v>שם_מקטע</v>
+      </c>
+      <c r="M165" t="str">
+        <v/>
+      </c>
+      <c r="N165" t="str">
+        <v>פרשת העקידה</v>
+      </c>
+      <c r="O165" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="166" xml:space="preserve">
+      <c r="A166" t="str">
+        <v>chg_1773733140069_rtmbazn</v>
+      </c>
+      <c r="B166" t="str">
+        <v>17.3.2026, 9:39:00</v>
+      </c>
+      <c r="C166" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D166" t="str">
+        <v>edot_mizrah</v>
+      </c>
+      <c r="E166" t="str">
+        <v>0-edot_mizrah</v>
+      </c>
+      <c r="F166" t="str">
+        <v/>
+      </c>
+      <c r="G166" t="str">
+        <v>3015010</v>
+      </c>
+      <c r="H166" t="str">
+        <v>3011035</v>
+      </c>
+      <c r="I166" t="str">
+        <v>3011035</v>
+      </c>
+      <c r="J166" t="str">
+        <v>301014711035</v>
+      </c>
+      <c r="K166" t="str">
+        <v>301014711035</v>
+      </c>
+      <c r="L166" t="str">
+        <v>content</v>
+      </c>
+      <c r="M166" t="str">
+        <v>בקשות</v>
+      </c>
+      <c r="N166" t="str" xml:space="preserve">
+        <v xml:space="preserve">בקשות
+-</v>
+      </c>
+      <c r="O166" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="str">
+        <v>chg_1773733142825_6uxc5ua</v>
+      </c>
+      <c r="B167" t="str">
+        <v>17.3.2026, 9:39:02</v>
+      </c>
+      <c r="C167" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D167" t="str">
+        <v>edot_mizrah</v>
+      </c>
+      <c r="E167" t="str">
+        <v/>
+      </c>
+      <c r="F167" t="str">
+        <v/>
+      </c>
+      <c r="G167" t="str">
+        <v/>
+      </c>
+      <c r="H167" t="str">
+        <v/>
+      </c>
+      <c r="I167" t="str">
+        <v/>
+      </c>
+      <c r="J167" t="str">
+        <v/>
+      </c>
+      <c r="K167" t="str">
+        <v/>
+      </c>
+      <c r="L167" t="str">
+        <v>פרסום</v>
+      </c>
+      <c r="M167" t="str">
+        <v/>
+      </c>
+      <c r="N167" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="O167" t="str">
+        <v>V</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O164"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O167"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
add names to excel
</commit_message>
<xml_diff>
--- a/docs/cms-changes.xlsx
+++ b/docs/cms-changes.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:O45"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1940,16 +1940,63 @@
         <v>כן</v>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>chg_1773736180069_q6pog39</v>
+      </c>
+      <c r="B45" t="str">
+        <v>17.3.2026, 10:29:40</v>
+      </c>
+      <c r="C45" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D45" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E45" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="F45" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="G45" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="H45" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="I45" t="str">
+        <v>שחרית</v>
+      </c>
+      <c r="J45" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="K45" t="str">
+        <v>השכמת הבוקר</v>
+      </c>
+      <c r="L45">
+        <v>1</v>
+      </c>
+      <c r="M45" t="str">
+        <v>1 שינוי שדה</v>
+      </c>
+      <c r="N45" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O45" t="str">
+        <v>לא</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K44"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O45"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O167"/>
+  <dimension ref="A1:P168"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -9801,9 +9848,59 @@
         <v>V</v>
       </c>
     </row>
+    <row r="168">
+      <c r="A168" t="str">
+        <v>chg_1773736180069_q6pog39</v>
+      </c>
+      <c r="B168" t="str">
+        <v>17.3.2026, 10:29:40</v>
+      </c>
+      <c r="C168" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D168" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E168" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F168" t="str">
+        <v/>
+      </c>
+      <c r="G168" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H168" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I168" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J168" t="str">
+        <v>101001411030</v>
+      </c>
+      <c r="K168" t="str">
+        <v>_שחרית_*</v>
+      </c>
+      <c r="L168" t="str">
+        <v>101001411030</v>
+      </c>
+      <c r="M168" t="str">
+        <v>content</v>
+      </c>
+      <c r="N168" t="str">
+        <v>_שחרית_**</v>
+      </c>
+      <c r="O168" t="str">
+        <v>_שחרית_*</v>
+      </c>
+      <c r="P168" t="str">
+        <v>V</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O167"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P168"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chnage to core from cloud firecms
</commit_message>
<xml_diff>
--- a/docs/cms-changes.xlsx
+++ b/docs/cms-changes.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O45"/>
+  <dimension ref="A1:O47"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1987,16 +1987,110 @@
         <v>לא</v>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>chg_1773740930839_bu3l3n1</v>
+      </c>
+      <c r="B46" t="str">
+        <v>17.3.2026, 11:48:50</v>
+      </c>
+      <c r="C46" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D46" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E46" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="F46" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="G46" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="H46" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="I46" t="str">
+        <v>שחרית</v>
+      </c>
+      <c r="J46" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="K46" t="str">
+        <v>השכמת הבוקר</v>
+      </c>
+      <c r="L46">
+        <v>1</v>
+      </c>
+      <c r="M46" t="str">
+        <v>1 שינוי שדה</v>
+      </c>
+      <c r="N46" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O46" t="str">
+        <v>לא</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>chg_1773740934411_senpq6p</v>
+      </c>
+      <c r="B47" t="str">
+        <v>17.3.2026, 11:48:54</v>
+      </c>
+      <c r="C47" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D47" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E47" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
+      <c r="H47" t="str">
+        <v/>
+      </c>
+      <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47" t="str">
+        <v/>
+      </c>
+      <c r="K47" t="str">
+        <v/>
+      </c>
+      <c r="L47">
+        <v>0</v>
+      </c>
+      <c r="M47" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="N47" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O47" t="str">
+        <v>כן</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O47"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P168"/>
+  <dimension ref="A1:P170"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -9898,9 +9992,109 @@
         <v>V</v>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" t="str">
+        <v>chg_1773740930839_bu3l3n1</v>
+      </c>
+      <c r="B169" t="str">
+        <v>17.3.2026, 11:48:50</v>
+      </c>
+      <c r="C169" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D169" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E169" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F169" t="str">
+        <v/>
+      </c>
+      <c r="G169" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H169" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I169" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J169" t="str">
+        <v>101001411030</v>
+      </c>
+      <c r="K169" t="str">
+        <v>_שחרית_*(</v>
+      </c>
+      <c r="L169" t="str">
+        <v>101001411030</v>
+      </c>
+      <c r="M169" t="str">
+        <v>content</v>
+      </c>
+      <c r="N169" t="str">
+        <v>_שחרית_*</v>
+      </c>
+      <c r="O169" t="str">
+        <v>_שחרית_*(</v>
+      </c>
+      <c r="P169" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="str">
+        <v>chg_1773740934411_senpq6p</v>
+      </c>
+      <c r="B170" t="str">
+        <v>17.3.2026, 11:48:54</v>
+      </c>
+      <c r="C170" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D170" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E170" t="str">
+        <v/>
+      </c>
+      <c r="F170" t="str">
+        <v/>
+      </c>
+      <c r="G170" t="str">
+        <v/>
+      </c>
+      <c r="H170" t="str">
+        <v/>
+      </c>
+      <c r="I170" t="str">
+        <v/>
+      </c>
+      <c r="J170" t="str">
+        <v/>
+      </c>
+      <c r="K170" t="str">
+        <v/>
+      </c>
+      <c r="L170" t="str">
+        <v/>
+      </c>
+      <c r="M170" t="str">
+        <v>פרסום</v>
+      </c>
+      <c r="N170" t="str">
+        <v/>
+      </c>
+      <c r="O170" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="P170" t="str">
+        <v>V</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P168"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P170"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
revert complex ids calculation
</commit_message>
<xml_diff>
--- a/docs/cms-changes.xlsx
+++ b/docs/cms-changes.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O134"/>
+  <dimension ref="A1:O143"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6170,16 +6170,439 @@
         <v/>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>chg_1774865601066_hrjgptk</v>
+      </c>
+      <c r="B135" t="str">
+        <v>30.3.2026, 13:13:21</v>
+      </c>
+      <c r="C135" t="str">
+        <v>update_toc</v>
+      </c>
+      <c r="D135" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E135" t="str">
+        <v>אשכנז</v>
+      </c>
+      <c r="F135" t="str">
+        <v/>
+      </c>
+      <c r="G135" t="str">
+        <v/>
+      </c>
+      <c r="H135" t="str">
+        <v/>
+      </c>
+      <c r="I135" t="str">
+        <v/>
+      </c>
+      <c r="J135" t="str">
+        <v/>
+      </c>
+      <c r="K135" t="str">
+        <v/>
+      </c>
+      <c r="L135">
+        <v>0</v>
+      </c>
+      <c r="M135" t="str">
+        <v>update_toc</v>
+      </c>
+      <c r="N135" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O135" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>chg_1774865613717_iglcbjj</v>
+      </c>
+      <c r="B136" t="str">
+        <v>30.3.2026, 13:13:33</v>
+      </c>
+      <c r="C136" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D136" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E136" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="F136" t="str">
+        <v/>
+      </c>
+      <c r="G136" t="str">
+        <v/>
+      </c>
+      <c r="H136" t="str">
+        <v/>
+      </c>
+      <c r="I136" t="str">
+        <v/>
+      </c>
+      <c r="J136" t="str">
+        <v/>
+      </c>
+      <c r="K136" t="str">
+        <v/>
+      </c>
+      <c r="L136">
+        <v>0</v>
+      </c>
+      <c r="M136" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="N136" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O136" t="str">
+        <v>כן</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>chg_1774877810749_1qosoo6</v>
+      </c>
+      <c r="B137" t="str">
+        <v>30.3.2026, 16:36:50</v>
+      </c>
+      <c r="C137" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D137" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E137" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="F137" t="str">
+        <v/>
+      </c>
+      <c r="G137" t="str">
+        <v/>
+      </c>
+      <c r="H137" t="str">
+        <v/>
+      </c>
+      <c r="I137" t="str">
+        <v/>
+      </c>
+      <c r="J137" t="str">
+        <v/>
+      </c>
+      <c r="K137" t="str">
+        <v/>
+      </c>
+      <c r="L137">
+        <v>0</v>
+      </c>
+      <c r="M137" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="N137" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O137" t="str">
+        <v>כן</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>chg_1774879565935_pjjyahz</v>
+      </c>
+      <c r="B138" t="str">
+        <v>30.3.2026, 17:06:05</v>
+      </c>
+      <c r="C138" t="str">
+        <v>create_translation_item</v>
+      </c>
+      <c r="D138" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E138" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="F138" t="str">
+        <v>1-ashkenaz</v>
+      </c>
+      <c r="G138" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="H138" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="I138" t="str">
+        <v>שחרית--</v>
+      </c>
+      <c r="J138" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="K138" t="str">
+        <v>השכמת הבוקר--</v>
+      </c>
+      <c r="L138">
+        <v>1</v>
+      </c>
+      <c r="M138" t="str">
+        <v>הוספת תרגום לפריט 101001498530</v>
+      </c>
+      <c r="N138" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O138" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>chg_1774879573904_47h1eta</v>
+      </c>
+      <c r="B139" t="str">
+        <v>30.3.2026, 17:06:13</v>
+      </c>
+      <c r="C139" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D139" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E139" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="F139" t="str">
+        <v/>
+      </c>
+      <c r="G139" t="str">
+        <v/>
+      </c>
+      <c r="H139" t="str">
+        <v/>
+      </c>
+      <c r="I139" t="str">
+        <v/>
+      </c>
+      <c r="J139" t="str">
+        <v/>
+      </c>
+      <c r="K139" t="str">
+        <v/>
+      </c>
+      <c r="L139">
+        <v>0</v>
+      </c>
+      <c r="M139" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="N139" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O139" t="str">
+        <v>כן</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="str">
+        <v>chg_1774880057659_rnwxooj</v>
+      </c>
+      <c r="B140" t="str">
+        <v>30.3.2026, 17:14:17</v>
+      </c>
+      <c r="C140" t="str">
+        <v>create_translation_item</v>
+      </c>
+      <c r="D140" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="E140" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="F140" t="str">
+        <v>1-sefard</v>
+      </c>
+      <c r="G140" t="str">
+        <v>0-sefard</v>
+      </c>
+      <c r="H140" t="str">
+        <v>2015010</v>
+      </c>
+      <c r="I140" t="str">
+        <v>שחרית</v>
+      </c>
+      <c r="J140" t="str">
+        <v>2011030</v>
+      </c>
+      <c r="K140" t="str">
+        <v>השכמת הבוקר--</v>
+      </c>
+      <c r="L140">
+        <v>1</v>
+      </c>
+      <c r="M140" t="str">
+        <v>הוספת תרגום לפריט 201002561030</v>
+      </c>
+      <c r="N140" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O140" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="str">
+        <v>chg_1774880062284_0sal5rh</v>
+      </c>
+      <c r="B141" t="str">
+        <v>30.3.2026, 17:14:22</v>
+      </c>
+      <c r="C141" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D141" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="E141" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="F141" t="str">
+        <v/>
+      </c>
+      <c r="G141" t="str">
+        <v/>
+      </c>
+      <c r="H141" t="str">
+        <v/>
+      </c>
+      <c r="I141" t="str">
+        <v/>
+      </c>
+      <c r="J141" t="str">
+        <v/>
+      </c>
+      <c r="K141" t="str">
+        <v/>
+      </c>
+      <c r="L141">
+        <v>0</v>
+      </c>
+      <c r="M141" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="N141" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O141" t="str">
+        <v>כן</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="str">
+        <v>chg_1774881518749_zzxay7q</v>
+      </c>
+      <c r="B142" t="str">
+        <v>30.3.2026, 17:38:38</v>
+      </c>
+      <c r="C142" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D142" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="E142" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="F142" t="str">
+        <v>0-sefard</v>
+      </c>
+      <c r="G142" t="str">
+        <v>0-sefard</v>
+      </c>
+      <c r="H142" t="str">
+        <v>2015010</v>
+      </c>
+      <c r="I142" t="str">
+        <v>שחרית</v>
+      </c>
+      <c r="J142" t="str">
+        <v>2011030</v>
+      </c>
+      <c r="K142" t="str">
+        <v>השכמת הבוקר--</v>
+      </c>
+      <c r="L142">
+        <v>2</v>
+      </c>
+      <c r="M142" t="str">
+        <v>2 שינוי שדה</v>
+      </c>
+      <c r="N142" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O142" t="str">
+        <v>לא</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="str">
+        <v>chg_1774881624954_4a3kblg</v>
+      </c>
+      <c r="B143" t="str">
+        <v>30.3.2026, 17:40:24</v>
+      </c>
+      <c r="C143" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D143" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="E143" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="F143" t="str">
+        <v/>
+      </c>
+      <c r="G143" t="str">
+        <v/>
+      </c>
+      <c r="H143" t="str">
+        <v/>
+      </c>
+      <c r="I143" t="str">
+        <v/>
+      </c>
+      <c r="J143" t="str">
+        <v/>
+      </c>
+      <c r="K143" t="str">
+        <v/>
+      </c>
+      <c r="L143">
+        <v>0</v>
+      </c>
+      <c r="M143" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="N143" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O143" t="str">
+        <v>כן</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O134"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O143"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P480"/>
+  <dimension ref="A1:P490"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -30081,9 +30504,509 @@
         <v>V</v>
       </c>
     </row>
+    <row r="481">
+      <c r="A481" t="str">
+        <v>chg_1774865601066_hrjgptk</v>
+      </c>
+      <c r="B481" t="str">
+        <v>30.3.2026, 13:13:21</v>
+      </c>
+      <c r="C481" t="str">
+        <v>update_toc</v>
+      </c>
+      <c r="D481" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E481" t="str">
+        <v/>
+      </c>
+      <c r="F481" t="str">
+        <v/>
+      </c>
+      <c r="G481" t="str">
+        <v/>
+      </c>
+      <c r="H481" t="str">
+        <v/>
+      </c>
+      <c r="I481" t="str">
+        <v/>
+      </c>
+      <c r="J481" t="str">
+        <v/>
+      </c>
+      <c r="K481" t="str">
+        <v/>
+      </c>
+      <c r="L481" t="str">
+        <v/>
+      </c>
+      <c r="M481" t="str">
+        <v>שם_נוסח</v>
+      </c>
+      <c r="N481" t="str">
+        <v/>
+      </c>
+      <c r="O481" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="P481" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="str">
+        <v>chg_1774865613717_iglcbjj</v>
+      </c>
+      <c r="B482" t="str">
+        <v>30.3.2026, 13:13:33</v>
+      </c>
+      <c r="C482" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D482" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E482" t="str">
+        <v/>
+      </c>
+      <c r="F482" t="str">
+        <v/>
+      </c>
+      <c r="G482" t="str">
+        <v/>
+      </c>
+      <c r="H482" t="str">
+        <v/>
+      </c>
+      <c r="I482" t="str">
+        <v/>
+      </c>
+      <c r="J482" t="str">
+        <v/>
+      </c>
+      <c r="K482" t="str">
+        <v/>
+      </c>
+      <c r="L482" t="str">
+        <v/>
+      </c>
+      <c r="M482" t="str">
+        <v>פרסום</v>
+      </c>
+      <c r="N482" t="str">
+        <v/>
+      </c>
+      <c r="O482" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="P482" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="str">
+        <v>chg_1774877810749_1qosoo6</v>
+      </c>
+      <c r="B483" t="str">
+        <v>30.3.2026, 16:36:50</v>
+      </c>
+      <c r="C483" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D483" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E483" t="str">
+        <v/>
+      </c>
+      <c r="F483" t="str">
+        <v/>
+      </c>
+      <c r="G483" t="str">
+        <v/>
+      </c>
+      <c r="H483" t="str">
+        <v/>
+      </c>
+      <c r="I483" t="str">
+        <v/>
+      </c>
+      <c r="J483" t="str">
+        <v/>
+      </c>
+      <c r="K483" t="str">
+        <v/>
+      </c>
+      <c r="L483" t="str">
+        <v/>
+      </c>
+      <c r="M483" t="str">
+        <v>פרסום</v>
+      </c>
+      <c r="N483" t="str">
+        <v/>
+      </c>
+      <c r="O483" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="P483" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="str">
+        <v>chg_1774879565935_pjjyahz</v>
+      </c>
+      <c r="B484" t="str">
+        <v>30.3.2026, 17:06:05</v>
+      </c>
+      <c r="C484" t="str">
+        <v>create_translation_item</v>
+      </c>
+      <c r="D484" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E484" t="str">
+        <v>1-ashkenaz</v>
+      </c>
+      <c r="F484" t="str">
+        <v/>
+      </c>
+      <c r="G484" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H484" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I484" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J484" t="str">
+        <v>121001661030</v>
+      </c>
+      <c r="K484" t="str">
+        <v>after</v>
+      </c>
+      <c r="L484" t="str">
+        <v>121001661030</v>
+      </c>
+      <c r="M484" t="str">
+        <v>פריט_תרגום</v>
+      </c>
+      <c r="N484" t="str">
+        <v/>
+      </c>
+      <c r="O484" t="str">
+        <v>121001661030</v>
+      </c>
+      <c r="P484" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="str">
+        <v>chg_1774879573904_47h1eta</v>
+      </c>
+      <c r="B485" t="str">
+        <v>30.3.2026, 17:06:13</v>
+      </c>
+      <c r="C485" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D485" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E485" t="str">
+        <v/>
+      </c>
+      <c r="F485" t="str">
+        <v/>
+      </c>
+      <c r="G485" t="str">
+        <v/>
+      </c>
+      <c r="H485" t="str">
+        <v/>
+      </c>
+      <c r="I485" t="str">
+        <v/>
+      </c>
+      <c r="J485" t="str">
+        <v/>
+      </c>
+      <c r="K485" t="str">
+        <v/>
+      </c>
+      <c r="L485" t="str">
+        <v/>
+      </c>
+      <c r="M485" t="str">
+        <v>פרסום</v>
+      </c>
+      <c r="N485" t="str">
+        <v/>
+      </c>
+      <c r="O485" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="P485" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="str">
+        <v>chg_1774880057659_rnwxooj</v>
+      </c>
+      <c r="B486" t="str">
+        <v>30.3.2026, 17:14:17</v>
+      </c>
+      <c r="C486" t="str">
+        <v>create_translation_item</v>
+      </c>
+      <c r="D486" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="E486" t="str">
+        <v>1-sefard</v>
+      </c>
+      <c r="F486" t="str">
+        <v/>
+      </c>
+      <c r="G486" t="str">
+        <v>2015010</v>
+      </c>
+      <c r="H486" t="str">
+        <v>2011030</v>
+      </c>
+      <c r="I486" t="str">
+        <v>2011030</v>
+      </c>
+      <c r="J486" t="str">
+        <v>221002549033</v>
+      </c>
+      <c r="K486" t="str">
+        <v>add sefarad</v>
+      </c>
+      <c r="L486" t="str">
+        <v>221002549033</v>
+      </c>
+      <c r="M486" t="str">
+        <v>פריט_תרגום</v>
+      </c>
+      <c r="N486" t="str">
+        <v/>
+      </c>
+      <c r="O486" t="str">
+        <v>221002549033</v>
+      </c>
+      <c r="P486" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="str">
+        <v>chg_1774880062284_0sal5rh</v>
+      </c>
+      <c r="B487" t="str">
+        <v>30.3.2026, 17:14:22</v>
+      </c>
+      <c r="C487" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D487" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="E487" t="str">
+        <v/>
+      </c>
+      <c r="F487" t="str">
+        <v/>
+      </c>
+      <c r="G487" t="str">
+        <v/>
+      </c>
+      <c r="H487" t="str">
+        <v/>
+      </c>
+      <c r="I487" t="str">
+        <v/>
+      </c>
+      <c r="J487" t="str">
+        <v/>
+      </c>
+      <c r="K487" t="str">
+        <v/>
+      </c>
+      <c r="L487" t="str">
+        <v/>
+      </c>
+      <c r="M487" t="str">
+        <v>פרסום</v>
+      </c>
+      <c r="N487" t="str">
+        <v/>
+      </c>
+      <c r="O487" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="P487" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="str">
+        <v>chg_1774881518749_zzxay7q</v>
+      </c>
+      <c r="B488" t="str">
+        <v>30.3.2026, 17:38:38</v>
+      </c>
+      <c r="C488" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D488" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="E488" t="str">
+        <v>0-sefard</v>
+      </c>
+      <c r="F488" t="str">
+        <v/>
+      </c>
+      <c r="G488" t="str">
+        <v>2015010</v>
+      </c>
+      <c r="H488" t="str">
+        <v>2011030</v>
+      </c>
+      <c r="I488" t="str">
+        <v>2011030</v>
+      </c>
+      <c r="J488" t="str">
+        <v>221002549033</v>
+      </c>
+      <c r="K488" t="str">
+        <v>add sefarad-</v>
+      </c>
+      <c r="L488" t="str">
+        <v>221002549033</v>
+      </c>
+      <c r="M488" t="str">
+        <v>content</v>
+      </c>
+      <c r="N488" t="str">
+        <v>add sefarad</v>
+      </c>
+      <c r="O488" t="str">
+        <v>add sefarad-</v>
+      </c>
+      <c r="P488" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="str">
+        <v>chg_1774881518749_zzxay7q</v>
+      </c>
+      <c r="B489" t="str">
+        <v>30.3.2026, 17:38:38</v>
+      </c>
+      <c r="C489" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D489" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="E489" t="str">
+        <v>0-sefard</v>
+      </c>
+      <c r="F489" t="str">
+        <v/>
+      </c>
+      <c r="G489" t="str">
+        <v>2015010</v>
+      </c>
+      <c r="H489" t="str">
+        <v>2011030</v>
+      </c>
+      <c r="I489" t="str">
+        <v>2011030</v>
+      </c>
+      <c r="J489" t="str">
+        <v>221002511030</v>
+      </c>
+      <c r="K489" t="str">
+        <v>Shaḥarit--</v>
+      </c>
+      <c r="L489" t="str">
+        <v>221002511030</v>
+      </c>
+      <c r="M489" t="str">
+        <v>content</v>
+      </c>
+      <c r="N489" t="str">
+        <v>Shaḥarit</v>
+      </c>
+      <c r="O489" t="str">
+        <v>Shaḥarit--</v>
+      </c>
+      <c r="P489" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="str">
+        <v>chg_1774881624954_4a3kblg</v>
+      </c>
+      <c r="B490" t="str">
+        <v>30.3.2026, 17:40:24</v>
+      </c>
+      <c r="C490" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="D490" t="str">
+        <v>sefard</v>
+      </c>
+      <c r="E490" t="str">
+        <v/>
+      </c>
+      <c r="F490" t="str">
+        <v/>
+      </c>
+      <c r="G490" t="str">
+        <v/>
+      </c>
+      <c r="H490" t="str">
+        <v/>
+      </c>
+      <c r="I490" t="str">
+        <v/>
+      </c>
+      <c r="J490" t="str">
+        <v/>
+      </c>
+      <c r="K490" t="str">
+        <v/>
+      </c>
+      <c r="L490" t="str">
+        <v/>
+      </c>
+      <c r="M490" t="str">
+        <v>פרסום</v>
+      </c>
+      <c r="N490" t="str">
+        <v/>
+      </c>
+      <c r="O490" t="str">
+        <v>publish_to_bagel</v>
+      </c>
+      <c r="P490" t="str">
+        <v>V</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P480"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P490"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix mitid at trunslation
</commit_message>
<xml_diff>
--- a/docs/cms-changes.xlsx
+++ b/docs/cms-changes.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -682,16 +682,157 @@
         <v>לא</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>chg_1775731560114_0t64jee</v>
+      </c>
+      <c r="B7" t="str">
+        <v>9.4.2026, 13:46:00</v>
+      </c>
+      <c r="C7" t="str">
+        <v>create_translation_item</v>
+      </c>
+      <c r="D7" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E7" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="F7" t="str">
+        <v>1-ashkenaz</v>
+      </c>
+      <c r="G7" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="H7" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="I7" t="str">
+        <v>שחרית</v>
+      </c>
+      <c r="J7" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="K7" t="str">
+        <v>השכמת הבוקר</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="str">
+        <v>הוספת תרגום לפריט 101002212031</v>
+      </c>
+      <c r="N7" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>chg_1775731706986_xflrkfl</v>
+      </c>
+      <c r="B8" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C8" t="str">
+        <v>delete_part_item</v>
+      </c>
+      <c r="D8" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E8" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="F8" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="G8" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="H8" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="I8" t="str">
+        <v>שחרית</v>
+      </c>
+      <c r="J8" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="K8" t="str">
+        <v>השכמת הבוקר</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="str">
+        <v>מחיקת פריט 101002212030</v>
+      </c>
+      <c r="N8" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B9" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C9" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D9" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E9" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="F9" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="G9" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="H9" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="I9" t="str">
+        <v>שחרית</v>
+      </c>
+      <c r="J9" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="K9" t="str">
+        <v>השכמת הבוקר</v>
+      </c>
+      <c r="L9">
+        <v>19</v>
+      </c>
+      <c r="M9" t="str">
+        <v>19 שינוי שדה</v>
+      </c>
+      <c r="N9" t="str">
+        <v>כן</v>
+      </c>
+      <c r="O9" t="str">
+        <v>לא</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O9"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P43"/>
+  <dimension ref="A1:P64"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2843,9 +2984,1059 @@
         <v>V</v>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>chg_1775731560114_0t64jee</v>
+      </c>
+      <c r="B44" t="str">
+        <v>9.4.2026, 13:46:00</v>
+      </c>
+      <c r="C44" t="str">
+        <v>create_translation_item</v>
+      </c>
+      <c r="D44" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E44" t="str">
+        <v>1-ashkenaz</v>
+      </c>
+      <c r="F44" t="str">
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H44" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I44" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J44" t="str">
+        <v>101002061030</v>
+      </c>
+      <c r="K44" t="str">
+        <v>trunslation</v>
+      </c>
+      <c r="L44" t="str">
+        <v>101002061030</v>
+      </c>
+      <c r="M44" t="str">
+        <v>פריט_תרגום</v>
+      </c>
+      <c r="N44" t="str">
+        <v/>
+      </c>
+      <c r="O44" t="str">
+        <v>101002061030</v>
+      </c>
+      <c r="P44" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>chg_1775731706986_xflrkfl</v>
+      </c>
+      <c r="B45" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C45" t="str">
+        <v>delete_part_item</v>
+      </c>
+      <c r="D45" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E45" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F45" t="str">
+        <v/>
+      </c>
+      <c r="G45" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H45" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I45" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J45" t="str">
+        <v>101002212030</v>
+      </c>
+      <c r="K45" t="str">
+        <v>הוספה אחרי מחיקה</v>
+      </c>
+      <c r="L45" t="str">
+        <v>101002212030</v>
+      </c>
+      <c r="M45" t="str">
+        <v>פריט</v>
+      </c>
+      <c r="N45" t="str">
+        <v>101002212030</v>
+      </c>
+      <c r="O45" t="str">
+        <v/>
+      </c>
+      <c r="P45" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B46" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C46" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D46" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E46" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F46" t="str">
+        <v/>
+      </c>
+      <c r="G46" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H46" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I46" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J46" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K46" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L46" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M46" t="str">
+        <v>content</v>
+      </c>
+      <c r="N46" t="str">
+        <v/>
+      </c>
+      <c r="O46" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="P46" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B47" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C47" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D47" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E47" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F47" t="str">
+        <v/>
+      </c>
+      <c r="G47" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H47" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I47" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J47" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K47" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L47" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M47" t="str">
+        <v>type</v>
+      </c>
+      <c r="N47" t="str">
+        <v/>
+      </c>
+      <c r="O47" t="str">
+        <v>body</v>
+      </c>
+      <c r="P47" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B48" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C48" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D48" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E48" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F48" t="str">
+        <v/>
+      </c>
+      <c r="G48" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H48" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I48" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J48" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K48" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L48" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M48" t="str">
+        <v>titleType</v>
+      </c>
+      <c r="N48" t="str">
+        <v/>
+      </c>
+      <c r="O48" t="str">
+        <v/>
+      </c>
+      <c r="P48" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B49" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C49" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D49" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E49" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F49" t="str">
+        <v/>
+      </c>
+      <c r="G49" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H49" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I49" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J49" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K49" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L49" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M49" t="str">
+        <v>title</v>
+      </c>
+      <c r="N49" t="str">
+        <v/>
+      </c>
+      <c r="O49" t="str">
+        <v/>
+      </c>
+      <c r="P49" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B50" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C50" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D50" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E50" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F50" t="str">
+        <v/>
+      </c>
+      <c r="G50" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H50" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I50" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J50" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K50" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L50" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M50" t="str">
+        <v>fontTanach</v>
+      </c>
+      <c r="N50" t="str">
+        <v/>
+      </c>
+      <c r="O50" t="str">
+        <v>false</v>
+      </c>
+      <c r="P50" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B51" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C51" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D51" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E51" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F51" t="str">
+        <v/>
+      </c>
+      <c r="G51" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H51" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I51" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J51" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K51" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L51" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M51" t="str">
+        <v>bold</v>
+      </c>
+      <c r="N51" t="str">
+        <v/>
+      </c>
+      <c r="O51" t="str">
+        <v>false</v>
+      </c>
+      <c r="P51" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B52" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C52" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D52" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E52" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F52" t="str">
+        <v/>
+      </c>
+      <c r="G52" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H52" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I52" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J52" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K52" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L52" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M52" t="str">
+        <v>centerAlign</v>
+      </c>
+      <c r="N52" t="str">
+        <v/>
+      </c>
+      <c r="O52" t="str">
+        <v>false</v>
+      </c>
+      <c r="P52" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B53" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C53" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D53" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E53" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F53" t="str">
+        <v/>
+      </c>
+      <c r="G53" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H53" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I53" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J53" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K53" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L53" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M53" t="str">
+        <v>lineLine</v>
+      </c>
+      <c r="N53" t="str">
+        <v/>
+      </c>
+      <c r="O53" t="str">
+        <v>false</v>
+      </c>
+      <c r="P53" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B54" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C54" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D54" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E54" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F54" t="str">
+        <v/>
+      </c>
+      <c r="G54" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H54" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I54" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J54" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K54" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L54" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M54" t="str">
+        <v>red</v>
+      </c>
+      <c r="N54" t="str">
+        <v/>
+      </c>
+      <c r="O54" t="str">
+        <v>false</v>
+      </c>
+      <c r="P54" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B55" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C55" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D55" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E55" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F55" t="str">
+        <v/>
+      </c>
+      <c r="G55" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H55" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I55" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J55" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K55" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L55" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M55" t="str">
+        <v>justifyBlock</v>
+      </c>
+      <c r="N55" t="str">
+        <v/>
+      </c>
+      <c r="O55" t="str">
+        <v>false</v>
+      </c>
+      <c r="P55" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B56" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C56" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D56" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E56" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F56" t="str">
+        <v/>
+      </c>
+      <c r="G56" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H56" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I56" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J56" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K56" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L56" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M56" t="str">
+        <v>noSpace</v>
+      </c>
+      <c r="N56" t="str">
+        <v/>
+      </c>
+      <c r="O56" t="str">
+        <v>false</v>
+      </c>
+      <c r="P56" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B57" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C57" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D57" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E57" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F57" t="str">
+        <v/>
+      </c>
+      <c r="G57" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H57" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I57" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J57" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K57" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L57" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M57" t="str">
+        <v>block</v>
+      </c>
+      <c r="N57" t="str">
+        <v/>
+      </c>
+      <c r="O57" t="str">
+        <v>false</v>
+      </c>
+      <c r="P57" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B58" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C58" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D58" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E58" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F58" t="str">
+        <v/>
+      </c>
+      <c r="G58" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H58" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I58" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J58" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K58" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L58" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M58" t="str">
+        <v>firstInPage</v>
+      </c>
+      <c r="N58" t="str">
+        <v/>
+      </c>
+      <c r="O58" t="str">
+        <v>false</v>
+      </c>
+      <c r="P58" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B59" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C59" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D59" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E59" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F59" t="str">
+        <v/>
+      </c>
+      <c r="G59" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H59" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I59" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J59" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K59" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L59" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M59" t="str">
+        <v>specialDate</v>
+      </c>
+      <c r="N59" t="str">
+        <v/>
+      </c>
+      <c r="O59" t="str">
+        <v>false</v>
+      </c>
+      <c r="P59" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B60" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C60" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D60" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E60" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F60" t="str">
+        <v/>
+      </c>
+      <c r="G60" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H60" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I60" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J60" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K60" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L60" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M60" t="str">
+        <v>role</v>
+      </c>
+      <c r="N60" t="str">
+        <v/>
+      </c>
+      <c r="O60" t="str">
+        <v/>
+      </c>
+      <c r="P60" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B61" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C61" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D61" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E61" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F61" t="str">
+        <v/>
+      </c>
+      <c r="G61" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H61" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I61" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J61" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K61" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L61" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M61" t="str">
+        <v>reference</v>
+      </c>
+      <c r="N61" t="str">
+        <v/>
+      </c>
+      <c r="O61" t="str">
+        <v/>
+      </c>
+      <c r="P61" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B62" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C62" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D62" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E62" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F62" t="str">
+        <v/>
+      </c>
+      <c r="G62" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H62" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I62" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J62" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K62" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L62" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M62" t="str">
+        <v>specialSign</v>
+      </c>
+      <c r="N62" t="str">
+        <v/>
+      </c>
+      <c r="O62" t="str">
+        <v/>
+      </c>
+      <c r="P62" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B63" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C63" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D63" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E63" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F63" t="str">
+        <v/>
+      </c>
+      <c r="G63" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H63" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I63" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J63" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K63" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L63" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M63" t="str">
+        <v>dateSetId</v>
+      </c>
+      <c r="N63" t="str">
+        <v/>
+      </c>
+      <c r="O63" t="str">
+        <v>100</v>
+      </c>
+      <c r="P63" t="str">
+        <v>V</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>chg_1775731706999_eb5dahm</v>
+      </c>
+      <c r="B64" t="str">
+        <v>9.4.2026, 13:48:26</v>
+      </c>
+      <c r="C64" t="str">
+        <v>save_part_items</v>
+      </c>
+      <c r="D64" t="str">
+        <v>ashkenaz</v>
+      </c>
+      <c r="E64" t="str">
+        <v>0-ashkenaz</v>
+      </c>
+      <c r="F64" t="str">
+        <v/>
+      </c>
+      <c r="G64" t="str">
+        <v>1015010</v>
+      </c>
+      <c r="H64" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="I64" t="str">
+        <v>1011030</v>
+      </c>
+      <c r="J64" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="K64" t="str">
+        <v>אחרי תיקון</v>
+      </c>
+      <c r="L64" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="M64" t="str">
+        <v>mit_id</v>
+      </c>
+      <c r="N64" t="str">
+        <v/>
+      </c>
+      <c r="O64" t="str">
+        <v>101001711030</v>
+      </c>
+      <c r="P64" t="str">
+        <v>V</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P43"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P64"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>